<commit_message>
added logs to debug
</commit_message>
<xml_diff>
--- a/testData/LoginData.xlsx
+++ b/testData/LoginData.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\K9IN\eclipse-workspacetest\Lookup\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD6BC5C5-6B40-4F7C-BD32-F184810CC55C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E32214C7-BD27-4D1F-B29A-954E74676CB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>Email</t>
   </si>
@@ -86,18 +86,11 @@
   <si>
     <t>xyz</t>
   </si>
-  <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>Fail</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -438,19 +431,19 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="29.109375"/>
-    <col min="2" max="2" customWidth="true" width="22.33203125"/>
-    <col min="3" max="3" customWidth="true" width="31.6640625"/>
+    <col min="1" max="1" width="29.109375" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="3" max="3" width="31.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -461,9 +454,6 @@
       <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s" s="0">
-        <v>12</v>
-      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -472,9 +462,6 @@
       <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s" s="0">
-        <v>13</v>
-      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -482,9 +469,6 @@
       </c>
       <c r="B4" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -492,9 +476,6 @@
       <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C5" t="s" s="0">
-        <v>13</v>
-      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -503,9 +484,6 @@
       <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6" t="s" s="0">
-        <v>12</v>
-      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -513,9 +491,6 @@
       </c>
       <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>